<commit_message>
Plantilla carga masiva de materiales v3
</commit_message>
<xml_diff>
--- a/src/assets/plantilla_materiales.xlsx
+++ b/src/assets/plantilla_materiales.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlfredoMamby\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\CycloNet\InOut\Frontend_Inout\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35431C21-7E53-4872-809A-E5B36B5CE924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D00DC821-2BE6-4048-A3E0-3B928B79EBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Materiales" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
   <si>
     <t>Nombre*</t>
   </si>
@@ -61,12 +61,6 @@
     <t>Ubicación</t>
   </si>
   <si>
-    <t>ID Categoría</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>Unidades</t>
   </si>
   <si>
@@ -125,6 +119,15 @@
   </si>
   <si>
     <t>Sitio 1</t>
+  </si>
+  <si>
+    <t>Condimento a base de puré de tomate, azúcar y vinagre. Uso principal: base para salsas o acompañamiento directo.</t>
+  </si>
+  <si>
+    <t>ID Categoría*</t>
+  </si>
+  <si>
+    <t>Salsa de tomate san jorge</t>
   </si>
 </sst>
 </file>
@@ -134,7 +137,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -153,6 +156,12 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -571,7 +580,7 @@
     <col min="9" max="9" width="9.5625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="31.5" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:9" ht="47.25" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -597,28 +606,36 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="3" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="E2" s="3">
-        <f>+D2</f>
+      <c r="A2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="6">
         <v>0</v>
       </c>
+      <c r="D2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="F2" s="7">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="G2" s="7">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>9</v>
+        <v>27</v>
+      </c>
+      <c r="I2" s="4">
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.5">
@@ -1806,10 +1823,11 @@
       <c r="I150" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I1 I2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:H1" numberStoredAsText="1"/>
   </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -1818,7 +1836,7 @@
           <x14:formula1>
             <xm:f>Configuración!$A$2:$A$20</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:E2</xm:sqref>
+          <xm:sqref>D2:E150</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1836,102 +1854,102 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>